<commit_message>
List A/B: new brands only (exclude the 1,202 sent on 30 Oct), one tab per sector
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TE8a9ptd2NGPUtY6iZfzkb
</commit_message>
<xml_diff>
--- a/reports/F1-PRIVATE-200M-FUNDING-VALUATION-NOT-FOUND-2026-10-30.xlsx
+++ b/reports/F1-PRIVATE-200M-FUNDING-VALUATION-NOT-FOUND-2026-10-30.xlsx
@@ -8,23 +8,19 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUMMARY" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MASTER LIST" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NOT ON YOUR SHEETS" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Software, Internet &amp; AI" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NEAR MISSES" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CURRENT F1 DEAL (SET ASIDE)" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CHECKED - LEFT OUT" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COULD NOT VERIFY" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Software, Internet &amp; AI" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NEAR MISSES" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CURRENT F1 DEAL (SET ASIDE)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CHECKED - LEFT OUT" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COULD NOT VERIFY" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SUMMARY'!$A$1:$B$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MASTER LIST'!$A$1:$AH$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'NOT ON YOUR SHEETS'!$A$1:$AH$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Software, Internet &amp; AI'!$A$1:$AI$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'NEAR MISSES'!$A$1:$M$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'CURRENT F1 DEAL (SET ASIDE)'!$A$1:$J$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'CHECKED - LEFT OUT'!$A$1:$M$182</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'COULD NOT VERIFY'!$A$1:$M$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SUMMARY'!$A$1:$B$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Software, Internet &amp; AI'!$A$1:$AI$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'NEAR MISSES'!$A$1:$M$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CURRENT F1 DEAL (SET ASIDE)'!$A$1:$J$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'CHECKED - LEFT OUT'!$A$1:$M$181</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'COULD NOT VERIFY'!$A$1:$M$68</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -452,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -491,7 +487,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>List B - USD 200M+ raised, valuation not found / not disclosed</t>
+          <t>List B - USD 200M+ raised, valuation not found / not disclosed (all new; none were in the 30 Oct unicorn workbook)</t>
         </is>
       </c>
     </row>
@@ -540,17 +536,19 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Near misses (private, but under USD 200M raised)</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="n">
-        <v>0</v>
+          <t>Layout</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>One tab per sector; each brand sits on the tab of the sector it operates in, ranked by Sector Rank, with its overall Outreach Priority across the whole list.</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Qualify but already have a current F1 deal (set aside)</t>
+          <t>Near misses (private, but under USD 200M raised)</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
@@ -560,714 +558,140 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Checked and left out (listed, acquired, defunct, majority-owned, under USD 200M)</t>
+          <t>Qualify but already have a current F1 deal (set aside)</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>181</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Could not be verified (separate tab, not in the main list)</t>
+          <t>Checked and left out (listed, acquired, defunct, majority-owned, under USD 200M)</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>67</v>
+        <v>180</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>How each company was verified</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Connector and research data can be wrong, so each test rests on independent sources: PRIVATE &amp; INDEPENDENT - CB Insights' current unicorn list where relevant, Wikipedia's exited-unicorn table, and up to 24 dated Google-News headlines per company (IPO / acquisition / shutdown / majority-owner queries) ruled on company by company; FUNDING USD 200M+ - Apollo funded-company filter looked up by website (website matched to the same company) or dated funding headlines; VALUATION - CB Insights, a dated news ruling or a research figure with a source (Valuation source column). Funding evidence and News evidence columns show what each row rests on. Amber = lower confidence or no relevant news (ranked lower).</t>
-        </is>
+          <t>Could not be verified (separate tab, not in the main list)</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>67</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>F1 sponsors set aside</t>
+          <t>How each company was verified</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Matched against the 2026 partner rosters of Formula 1 and all 11 teams (424 deals) plus research.</t>
+          <t>Connector and research data can be wrong, so each test rests on independent sources: PRIVATE &amp; INDEPENDENT - CB Insights' current unicorn list where relevant, Wikipedia's exited-unicorn table, and up to 24 dated Google-News headlines per company (IPO / acquisition / shutdown / majority-owner queries) ruled on company by company; FUNDING USD 200M+ - Apollo funded-company filter looked up by website (website matched to the same company) or dated funding headlines; VALUATION - CB Insights, a dated news ruling or a research figure with a source (Valuation source column). Funding evidence and News evidence columns show what each row rests on. Amber = lower confidence or no relevant news (ranked lower).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Outreach order</t>
+          <t>F1 sponsors set aside</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Ranked by Outreach Priority = Total score + timing (fresh round, expansion or IPO prep, new marketing leadership, a rival already in F1) minus a penalty for lower-confidence rows. Tier 1 = top 150, Tier 2 = 151-500, Tier 3 = the rest. Sector tabs keep the same order.</t>
+          <t>Matched against the 2026 partner rosters of Formula 1 and all 11 teams (424 deals) plus research.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Scoring</t>
+          <t>Outreach order</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Total /100 = F1 Fit /60 (audience overlap, commercial synergies, brand alignment, international relevance, plus signals: rival in F1, motorsport link, expansion moment, race-market footprint, founder affinity) + Financial Capacity /40 (valuation and funding bands, headcount, funding recency, marketing hires, revenue).</t>
+          <t>Ranked by Outreach Priority = Total score + timing (fresh round, expansion or IPO prep, new marketing leadership, a rival already in F1) minus a penalty for lower-confidence rows. Tier 1 = top 150, Tier 2 = 151-500, Tier 3 = the rest. Sector tabs keep the same order.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Already on your sheets?</t>
+          <t>Scoring</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Checked against every name and website on MASTER REFERENCE OCT and the 2,000 F1 SPONSORSHIP PARENT COMPANY PROSPECTS workbook. Kept and flagged; the NOT ON YOUR SHEETS tab leaves them out.</t>
+          <t>Total /100 = F1 Fit /60 (audience overlap, commercial synergies, brand alignment, international relevance, plus signals: rival in F1, motorsport link, expansion moment, race-market footprint, founder affinity) + Financial Capacity /40 (valuation and funding bands, headcount, funding recency, marketing hires, revenue).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>Already on your sheets?</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Checked against every name and website on MASTER REFERENCE OCT and the 2,000 F1 SPONSORSHIP PARENT COMPANY PROSPECTS workbook. Kept and flagged; the NOT ON YOUR SHEETS tab leaves them out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>Sources</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Research agents across every sector and region (knowledge, Dealroom / Crunchbase News / Wikipedia pages and Google News), CB Insights and Wikipedia unicorn tables, Apollo funded-company database (free lookup, total funding USD 200M+) and Clay, Google News headlines, F1 team partner pages. Crunchbase's data allowance was exhausted until 1 Nov 2026 and Lusha / Apollo paid credits were used up, so their free tools were used.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr"/>
-      <c r="B18" s="2" t="inlineStr"/>
-    </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr"/>
+      <c r="B19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>HQ country: USA</t>
         </is>
       </c>
-      <c r="B19" s="2" t="n">
+      <c r="B20" s="2" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr"/>
-      <c r="B20" s="2" t="inlineStr"/>
-    </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr"/>
+      <c r="B21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>Sector: Software, Internet &amp; AI</t>
         </is>
       </c>
-      <c r="B21" s="2" t="n">
+      <c r="B22" s="2" t="n">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B21"/>
+  <autoFilter ref="A1:B22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:AH2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="38" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="38" customWidth="1" min="14" max="14"/>
-    <col width="30" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="9" customWidth="1" min="17" max="17"/>
-    <col width="18" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
-    <col width="38" customWidth="1" min="20" max="20"/>
-    <col width="42" customWidth="1" min="21" max="21"/>
-    <col width="8" customWidth="1" min="22" max="22"/>
-    <col width="8" customWidth="1" min="23" max="23"/>
-    <col width="8" customWidth="1" min="24" max="24"/>
-    <col width="8" customWidth="1" min="25" max="25"/>
-    <col width="30" customWidth="1" min="26" max="26"/>
-    <col width="22" customWidth="1" min="27" max="27"/>
-    <col width="42" customWidth="1" min="28" max="28"/>
-    <col width="9" customWidth="1" min="29" max="29"/>
-    <col width="40" customWidth="1" min="30" max="30"/>
-    <col width="11" customWidth="1" min="31" max="31"/>
-    <col width="40" customWidth="1" min="32" max="32"/>
-    <col width="30" customWidth="1" min="33" max="33"/>
-    <col width="14" customWidth="1" min="34" max="34"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Outreach Priority</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Tier</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Brand</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>HQ Country</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>HQ City</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Website</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Industry / Sector</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>What they do</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Valuation (USD bn)</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Valuation date</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Valuation band</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Valuation source</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Total Funding (USD M)</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Latest round</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Top investors</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Revenue / ARR (USD M)</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>New unicorn 2025-26</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Already on your sheets?</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>On 30 Oct new-brands list?</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>Why contact now</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>Why F1 fits</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>Priority score</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>F1 Fit (/60)</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>Financial Capacity (/40)</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>Total (/100)</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>Other sport deals</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>CEO / founder</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>Signal evidence</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>Research confidence</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>Funding evidence</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>News check</t>
-        </is>
-      </c>
-      <c r="AF1" s="1" t="inlineStr">
-        <is>
-          <t>News evidence / source</t>
-        </is>
-      </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="AH1" s="1" t="inlineStr">
-        <is>
-          <t>Found by</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Tier 1 - contact first</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Suki</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>Redwood City</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>https://suki.ai</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>Software, Internet &amp; AI</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>AI voice assistant for physicians</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>not disclosed</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr"/>
-      <c r="K2" s="3" t="inlineStr">
-        <is>
-          <t>Valuation not disclosed</t>
-        </is>
-      </c>
-      <c r="L2" s="3" t="inlineStr"/>
-      <c r="M2" s="3" t="inlineStr"/>
-      <c r="N2" s="3" t="inlineStr">
-        <is>
-          <t>Series E USD 90M, Oct 2026</t>
-        </is>
-      </c>
-      <c r="O2" s="3" t="inlineStr">
-        <is>
-          <t>Healthier Capital, Crosslink</t>
-        </is>
-      </c>
-      <c r="P2" s="3" t="inlineStr"/>
-      <c r="Q2" s="3" t="inlineStr"/>
-      <c r="R2" s="3" t="inlineStr">
-        <is>
-          <t>yes (website match)</t>
-        </is>
-      </c>
-      <c r="S2" s="3" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="T2" s="3" t="inlineStr">
-        <is>
-          <t>fresh round in 2025-26</t>
-        </is>
-      </c>
-      <c r="U2" s="3" t="inlineStr">
-        <is>
-          <t>Valuation undisclosed.</t>
-        </is>
-      </c>
-      <c r="V2" s="3" t="n">
-        <v>23.3</v>
-      </c>
-      <c r="W2" s="3" t="n">
-        <v>16.3</v>
-      </c>
-      <c r="X2" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="Y2" s="3" t="n">
-        <v>25.3</v>
-      </c>
-      <c r="Z2" s="3" t="inlineStr"/>
-      <c r="AA2" s="3" t="inlineStr">
-        <is>
-          <t>Punit Soni</t>
-        </is>
-      </c>
-      <c r="AB2" s="3" t="inlineStr">
-        <is>
-          <t>Series E Oct 2026.</t>
-        </is>
-      </c>
-      <c r="AC2" s="3" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="AD2" s="3" t="inlineStr">
-        <is>
-          <t>Apollo: total funding &gt;= USD 200M</t>
-        </is>
-      </c>
-      <c r="AE2" s="3" t="inlineStr">
-        <is>
-          <t>unconfirmed by news</t>
-        </is>
-      </c>
-      <c r="AF2" s="3" t="inlineStr">
-        <is>
-          <t>Exclusive: Ambient scribe startup Suki raises $90M Series E - Axios (12 Oct 2026)</t>
-        </is>
-      </c>
-      <c r="AG2" s="3" t="inlineStr">
-        <is>
-          <t>Valuation not found.</t>
-        </is>
-      </c>
-      <c r="AH2" s="3" t="inlineStr">
-        <is>
-          <t>u06</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:AH2"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:AH1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="38" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="38" customWidth="1" min="14" max="14"/>
-    <col width="30" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="9" customWidth="1" min="17" max="17"/>
-    <col width="18" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
-    <col width="38" customWidth="1" min="20" max="20"/>
-    <col width="42" customWidth="1" min="21" max="21"/>
-    <col width="8" customWidth="1" min="22" max="22"/>
-    <col width="8" customWidth="1" min="23" max="23"/>
-    <col width="8" customWidth="1" min="24" max="24"/>
-    <col width="8" customWidth="1" min="25" max="25"/>
-    <col width="30" customWidth="1" min="26" max="26"/>
-    <col width="22" customWidth="1" min="27" max="27"/>
-    <col width="42" customWidth="1" min="28" max="28"/>
-    <col width="9" customWidth="1" min="29" max="29"/>
-    <col width="40" customWidth="1" min="30" max="30"/>
-    <col width="11" customWidth="1" min="31" max="31"/>
-    <col width="40" customWidth="1" min="32" max="32"/>
-    <col width="30" customWidth="1" min="33" max="33"/>
-    <col width="14" customWidth="1" min="34" max="34"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Outreach Priority</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Tier</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Brand</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>HQ Country</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>HQ City</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Website</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Industry / Sector</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>What they do</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Valuation (USD bn)</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Valuation date</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Valuation band</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Valuation source</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Total Funding (USD M)</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Latest round</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Top investors</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Revenue / ARR (USD M)</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>New unicorn 2025-26</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Already on your sheets?</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>On 30 Oct new-brands list?</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>Why contact now</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>Why F1 fits</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>Priority score</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>F1 Fit (/60)</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>Financial Capacity (/40)</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>Total (/100)</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>Other sport deals</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>CEO / founder</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>Signal evidence</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>Research confidence</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>Funding evidence</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>News check</t>
-        </is>
-      </c>
-      <c r="AF1" s="1" t="inlineStr">
-        <is>
-          <t>News evidence / source</t>
-        </is>
-      </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="AH1" s="1" t="inlineStr">
-        <is>
-          <t>Found by</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:AH1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1637,7 +1061,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1734,7 +1158,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1813,13 +1237,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M182"/>
+  <dimension ref="A1:M181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -11717,35 +11141,39 @@
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>Zip Co</t>
+          <t>eToro</t>
         </is>
       </c>
       <c r="B180" s="2" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Israel</t>
         </is>
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>https://zip.co</t>
+          <t>https://etoro.com</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>Financial Services &amp; Payments</t>
+          <t>Investment &amp; Capital Markets</t>
         </is>
       </c>
       <c r="E180" s="2" t="inlineStr">
         <is>
-          <t>Buy-now-pay-later provider</t>
+          <t>Social trading and investing platform</t>
         </is>
       </c>
       <c r="F180" s="2" t="inlineStr"/>
-      <c r="G180" s="2" t="inlineStr"/>
+      <c r="G180" s="2" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
       <c r="H180" s="2" t="inlineStr"/>
       <c r="I180" s="2" t="inlineStr">
         <is>
-          <t>Listed ASX</t>
+          <t>IPO Nasdaq May 2025 (ETOR)</t>
         </is>
       </c>
       <c r="J180" s="2" t="inlineStr">
@@ -11760,7 +11188,7 @@
       </c>
       <c r="L180" s="2" t="inlineStr">
         <is>
-          <t>ASX: ZIP</t>
+          <t>Israel HQ; listed May 2025.</t>
         </is>
       </c>
       <c r="M180" s="2" t="inlineStr"/>
@@ -11768,128 +11196,73 @@
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>eToro</t>
+          <t>ofo</t>
         </is>
       </c>
       <c r="B181" s="2" t="inlineStr">
         <is>
-          <t>Israel</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>https://etoro.com</t>
+          <t>https://ofo.com</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr">
         <is>
-          <t>Investment &amp; Capital Markets</t>
+          <t>Automotive &amp; Mobility</t>
         </is>
       </c>
       <c r="E181" s="2" t="inlineStr">
         <is>
-          <t>Social trading and investing platform</t>
-        </is>
-      </c>
-      <c r="F181" s="2" t="inlineStr"/>
+          <t>Failed bike-sharing startup</t>
+        </is>
+      </c>
+      <c r="F181" s="2" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
       <c r="G181" s="2" t="inlineStr">
         <is>
-          <t>2025-05</t>
-        </is>
-      </c>
-      <c r="H181" s="2" t="inlineStr"/>
+          <t>2018-03</t>
+        </is>
+      </c>
+      <c r="H181" s="2" t="inlineStr">
+        <is>
+          <t>2,200</t>
+        </is>
+      </c>
       <c r="I181" s="2" t="inlineStr">
         <is>
-          <t>IPO Nasdaq May 2025 (ETOR)</t>
+          <t>Series E+ 2018, Alibaba-led</t>
         </is>
       </c>
       <c r="J181" s="2" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>defunct</t>
         </is>
       </c>
       <c r="K181" s="2" t="inlineStr">
         <is>
-          <t>research: public | no valuation found | no funding figure (Apollo not checked)</t>
+          <t>research: defunct | research USD 2.00B (2018-03), not on CB Insights list | research ~USD 2,200M only (Apollo not checked)</t>
         </is>
       </c>
       <c r="L181" s="2" t="inlineStr">
         <is>
-          <t>Israel HQ; listed May 2025.</t>
+          <t>Defunct, excluded.</t>
         </is>
       </c>
       <c r="M181" s="2" t="inlineStr"/>
     </row>
-    <row r="182">
-      <c r="A182" s="2" t="inlineStr">
-        <is>
-          <t>ofo</t>
-        </is>
-      </c>
-      <c r="B182" s="2" t="inlineStr">
-        <is>
-          <t>China</t>
-        </is>
-      </c>
-      <c r="C182" s="2" t="inlineStr">
-        <is>
-          <t>https://ofo.com</t>
-        </is>
-      </c>
-      <c r="D182" s="2" t="inlineStr">
-        <is>
-          <t>Automotive &amp; Mobility</t>
-        </is>
-      </c>
-      <c r="E182" s="2" t="inlineStr">
-        <is>
-          <t>Failed bike-sharing startup</t>
-        </is>
-      </c>
-      <c r="F182" s="2" t="inlineStr">
-        <is>
-          <t>2.0</t>
-        </is>
-      </c>
-      <c r="G182" s="2" t="inlineStr">
-        <is>
-          <t>2018-03</t>
-        </is>
-      </c>
-      <c r="H182" s="2" t="inlineStr">
-        <is>
-          <t>2,200</t>
-        </is>
-      </c>
-      <c r="I182" s="2" t="inlineStr">
-        <is>
-          <t>Series E+ 2018, Alibaba-led</t>
-        </is>
-      </c>
-      <c r="J182" s="2" t="inlineStr">
-        <is>
-          <t>defunct</t>
-        </is>
-      </c>
-      <c r="K182" s="2" t="inlineStr">
-        <is>
-          <t>research: defunct | research USD 2.00B (2018-03), not on CB Insights list | research ~USD 2,200M only (Apollo not checked)</t>
-        </is>
-      </c>
-      <c r="L182" s="2" t="inlineStr">
-        <is>
-          <t>Defunct, excluded.</t>
-        </is>
-      </c>
-      <c r="M182" s="2" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:M182"/>
+  <autoFilter ref="A1:M181"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>